<commit_message>
Step 1: merge sheets and compute Abbott-corrected mortality
</commit_message>
<xml_diff>
--- a/analysis_outputs/step_01/Table_04_Step1_Summary_Check.xlsx
+++ b/analysis_outputs/step_01/Table_04_Step1_Summary_Check.xlsx
@@ -528,7 +528,7 @@
         <v>24</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H2" t="n">
         <v>11.25</v>
@@ -888,7 +888,7 @@
         <v>48</v>
       </c>
       <c r="G9" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H9" t="n">
         <v>11.25</v>
@@ -1248,7 +1248,7 @@
         <v>72</v>
       </c>
       <c r="G16" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H16" t="n">
         <v>11.25</v>
@@ -1608,7 +1608,7 @@
         <v>24</v>
       </c>
       <c r="G23" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H23" t="n">
         <v>52</v>
@@ -1968,7 +1968,7 @@
         <v>48</v>
       </c>
       <c r="G30" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H30" t="n">
         <v>52</v>
@@ -2328,7 +2328,7 @@
         <v>72</v>
       </c>
       <c r="G37" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H37" t="n">
         <v>52</v>
@@ -2688,7 +2688,7 @@
         <v>24</v>
       </c>
       <c r="G44" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H44" t="n">
         <v>59</v>
@@ -3048,7 +3048,7 @@
         <v>48</v>
       </c>
       <c r="G51" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H51" t="n">
         <v>59</v>
@@ -3408,7 +3408,7 @@
         <v>72</v>
       </c>
       <c r="G58" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H58" t="n">
         <v>59</v>
@@ -3768,7 +3768,7 @@
         <v>24</v>
       </c>
       <c r="G65" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H65" t="n">
         <v>9.5</v>
@@ -4128,7 +4128,7 @@
         <v>48</v>
       </c>
       <c r="G72" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H72" t="n">
         <v>9.5</v>
@@ -4488,7 +4488,7 @@
         <v>72</v>
       </c>
       <c r="G79" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H79" t="n">
         <v>9.5</v>
@@ -4848,7 +4848,7 @@
         <v>24</v>
       </c>
       <c r="G86" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H86" t="n">
         <v>49.5</v>
@@ -5208,7 +5208,7 @@
         <v>48</v>
       </c>
       <c r="G93" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H93" t="n">
         <v>49.5</v>
@@ -5568,7 +5568,7 @@
         <v>72</v>
       </c>
       <c r="G100" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H100" t="n">
         <v>49.5</v>
@@ -5928,7 +5928,7 @@
         <v>24</v>
       </c>
       <c r="G107" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H107" t="n">
         <v>54.25</v>
@@ -6288,7 +6288,7 @@
         <v>48</v>
       </c>
       <c r="G114" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H114" t="n">
         <v>54.25</v>
@@ -6648,7 +6648,7 @@
         <v>72</v>
       </c>
       <c r="G121" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H121" t="n">
         <v>54.25</v>
@@ -7008,7 +7008,7 @@
         <v>24</v>
       </c>
       <c r="G128" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H128" t="n">
         <v>10.25</v>
@@ -7368,7 +7368,7 @@
         <v>48</v>
       </c>
       <c r="G135" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H135" t="n">
         <v>10.25</v>
@@ -7728,7 +7728,7 @@
         <v>72</v>
       </c>
       <c r="G142" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H142" t="n">
         <v>10.25</v>
@@ -8088,7 +8088,7 @@
         <v>24</v>
       </c>
       <c r="G149" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H149" t="n">
         <v>51.75</v>
@@ -8448,7 +8448,7 @@
         <v>48</v>
       </c>
       <c r="G156" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H156" t="n">
         <v>51.75</v>
@@ -8808,7 +8808,7 @@
         <v>72</v>
       </c>
       <c r="G163" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H163" t="n">
         <v>51.75</v>
@@ -9168,7 +9168,7 @@
         <v>24</v>
       </c>
       <c r="G170" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H170" t="n">
         <v>56.75</v>
@@ -9528,7 +9528,7 @@
         <v>48</v>
       </c>
       <c r="G177" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H177" t="n">
         <v>56.75</v>
@@ -9888,7 +9888,7 @@
         <v>72</v>
       </c>
       <c r="G184" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H184" t="n">
         <v>56.75</v>
@@ -10248,7 +10248,7 @@
         <v>24</v>
       </c>
       <c r="G191" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H191" t="n">
         <v>11.25</v>
@@ -10608,7 +10608,7 @@
         <v>48</v>
       </c>
       <c r="G198" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H198" t="n">
         <v>11.25</v>
@@ -10968,7 +10968,7 @@
         <v>72</v>
       </c>
       <c r="G205" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H205" t="n">
         <v>11.25</v>
@@ -11328,7 +11328,7 @@
         <v>24</v>
       </c>
       <c r="G212" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H212" t="n">
         <v>57.5</v>
@@ -11688,7 +11688,7 @@
         <v>48</v>
       </c>
       <c r="G219" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H219" t="n">
         <v>57.5</v>
@@ -12048,7 +12048,7 @@
         <v>72</v>
       </c>
       <c r="G226" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H226" t="n">
         <v>57.5</v>
@@ -12408,7 +12408,7 @@
         <v>24</v>
       </c>
       <c r="G233" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H233" t="n">
         <v>63.5</v>
@@ -12768,7 +12768,7 @@
         <v>48</v>
       </c>
       <c r="G240" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H240" t="n">
         <v>63.5</v>
@@ -13128,7 +13128,7 @@
         <v>72</v>
       </c>
       <c r="G247" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H247" t="n">
         <v>63.5</v>
@@ -13488,7 +13488,7 @@
         <v>24</v>
       </c>
       <c r="G254" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H254" t="n">
         <v>9.5</v>
@@ -13848,7 +13848,7 @@
         <v>48</v>
       </c>
       <c r="G261" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H261" t="n">
         <v>9.5</v>
@@ -14208,7 +14208,7 @@
         <v>72</v>
       </c>
       <c r="G268" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H268" t="n">
         <v>9.5</v>
@@ -14568,7 +14568,7 @@
         <v>24</v>
       </c>
       <c r="G275" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H275" t="n">
         <v>50.25</v>
@@ -14928,7 +14928,7 @@
         <v>48</v>
       </c>
       <c r="G282" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H282" t="n">
         <v>50.25</v>
@@ -15288,7 +15288,7 @@
         <v>72</v>
       </c>
       <c r="G289" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H289" t="n">
         <v>50.25</v>
@@ -15648,7 +15648,7 @@
         <v>24</v>
       </c>
       <c r="G296" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H296" t="n">
         <v>54.75</v>
@@ -16008,7 +16008,7 @@
         <v>48</v>
       </c>
       <c r="G303" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H303" t="n">
         <v>54.75</v>
@@ -16368,7 +16368,7 @@
         <v>72</v>
       </c>
       <c r="G310" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H310" t="n">
         <v>54.75</v>
@@ -16728,7 +16728,7 @@
         <v>24</v>
       </c>
       <c r="G317" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H317" t="n">
         <v>10.75</v>
@@ -17088,7 +17088,7 @@
         <v>48</v>
       </c>
       <c r="G324" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H324" t="n">
         <v>10.75</v>
@@ -17448,7 +17448,7 @@
         <v>72</v>
       </c>
       <c r="G331" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H331" t="n">
         <v>10.75</v>
@@ -17808,7 +17808,7 @@
         <v>24</v>
       </c>
       <c r="G338" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H338" t="n">
         <v>68.5</v>
@@ -18168,7 +18168,7 @@
         <v>48</v>
       </c>
       <c r="G345" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H345" t="n">
         <v>68.5</v>
@@ -18528,7 +18528,7 @@
         <v>72</v>
       </c>
       <c r="G352" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H352" t="n">
         <v>68.5</v>
@@ -18888,7 +18888,7 @@
         <v>24</v>
       </c>
       <c r="G359" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H359" t="n">
         <v>70</v>
@@ -19248,7 +19248,7 @@
         <v>48</v>
       </c>
       <c r="G366" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H366" t="n">
         <v>70</v>
@@ -19608,7 +19608,7 @@
         <v>72</v>
       </c>
       <c r="G373" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H373" t="n">
         <v>70</v>

</xml_diff>